<commit_message>
Make deck a single source of truth: plan-data.json
Deck now fetches plan-data.json at runtime and computes revenue,
EBITDA, budget totals and breakeven client-side — matches the
formulas in scripts/build-plan-xlsx.py. To update numbers: edit
plan-data.json, then run `python3 scripts/build-plan-xlsx.py` to
regenerate the downloadable xlsx. Both the deck and xlsx stay in
sync from that one edit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plan/bookimmo_business_plan_v2.xlsx
+++ b/public/plan/bookimmo_business_plan_v2.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Model" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget Apr-Aug (USD 30K)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget Apr-Aug (USD)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Plan Sep+12M" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -41,7 +41,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,11 +51,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -81,20 +76,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -461,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -471,7 +462,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>book.immo — Business Model v2 (Sep 2026)</t>
+          <t>book.immo — Business Model v2</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -511,7 +502,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Локальные агентства подключают свои CRM к book.immo. Размещение БЕСПЛАТНО (агрегаторы берут деньги). Взамен — сплит комиссии при сделке.</t>
+          <t>Локальные агентства подключают свои CRM к book.immo. Размещение БЕСПЛАТНО. Взамен — сплит комиссии при сделке.</t>
         </is>
       </c>
     </row>
@@ -523,7 +514,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Объекты попадают к нам из CRM ДО публикации на агрегаторах (агентства платят агрегаторам за размещение и делают это с задержкой). Эксклюзивы — в топе выдачи по гео.</t>
+          <t>Объекты попадают к нам из CRM ДО публикации на агрегаторах. Эксклюзивы — в топе выдачи по гео.</t>
         </is>
       </c>
     </row>
@@ -547,7 +538,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Арендаторы/покупатели получают умный подбор + ИИ-автоматизацию: ИИ сам пишет письма, рассылает заявки, отслеживает новые объекты.</t>
+          <t>Арендаторы/покупатели получают умный подбор + ИИ-автоматизацию: заявки, мониторинг, документы.</t>
         </is>
       </c>
     </row>
@@ -559,7 +550,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Сделка закрывается агентством → комиссия делится между book.immo и маклером. Плюс pay-per-result ИИ-сервисы.</t>
+          <t>Сделку закрывает агентство → комиссия делится между book.immo и маклером. Плюс pay-per-result ИИ-сервисы.</t>
         </is>
       </c>
     </row>
@@ -571,7 +562,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Zolak.tech (virtual staging), ИИ-экспозе, квалифицированные лиды из нашей B2C-базы.</t>
+          <t>Zolak.tech (virtual staging), ИИ-экспозе, квалифицированные лиды из B2C-базы.</t>
         </is>
       </c>
     </row>
@@ -581,7 +572,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3">
-        <f>== REVENUE STREAMS ===</f>
+        <f>== LEGAL ===</f>
         <v/>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
@@ -589,166 +580,48 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R1. Сплит аренда</t>
+          <t>Wohnungsvermittlungsgesetz</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Маклер получает ~2 Kaltmieten (~EUR 2,000-2,400) с собственника (Bestellerprinzip). Доля book.immo 25-30% = ~EUR 600/сделка.</t>
+          <t>Нельзя брать с арендатора комиссию за посредничество аренды. B2C fee — плата за софт, не за посредничество.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R2. Сплит продажа</t>
+          <t>Bestellerprinzip</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Tippgeberprovision 20% от комиссии маклера (~EUR 12,000 при цене EUR 400K x 3%) = ~EUR 2,400/сделка.</t>
+          <t>Комиссию платит собственник маклеру. Сплит book.immo — из B2B-агентского договора. Легально.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R3. B2C AI-сервисы</t>
+          <t>GDPR</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Success fee EUR 149 за подписанный договор через ИИ-автоплатформу (заявки, мониторинг, документы). Оформлено как ТЕХНОЛОГИЧЕСКИЙ сервис, не посредничество.</t>
+          <t>DPA-договоры с агентствами; consent B2C-клиентов на передачу заявки.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R4. Agency upsells (позже)</t>
+          <t>Парсинг</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Zolak staging, ИИ-экспозе, premium-размещение лидов — аффилиат/маржа. С M6+.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3">
-        <f>== LEGAL (критично) ===</f>
-        <v/>
-      </c>
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Wohnungsvermittlungsgesetz</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>НЕЛЬЗЯ брать с арендатора комиссию за посредничество аренды. B2C-монетизация = плата за софт/автоматизацию (SaaS/success fee за сервис), договор без слова "Vermittlung".</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Bestellerprinzip</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Комиссию за аренду платит заказчик (собственник) маклеру. Наш сплит — из комиссии маклера по агентскому договору B2B. Легально.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>GDPR</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Данные из CRM агентств — DPA-договоры с каждым агентством, данные B2C-клиентов — consent на передачу агентству.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Парсинг</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Публичные витрины; соблюдать robots/ToS-риски, не публиковать чужие фото без обработки. Риск-менеджмент: эксклюзивы снижают зависимость от парсинга.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3">
-        <f>== MOAT / отличие от агрегаторов ===</f>
-        <v/>
-      </c>
-      <c r="B25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Время</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Pre-market инвентарь: доступ к объектам до агрегаторов = главный магнит для B2C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Цена для агентств</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>0 EUR размещение против EUR 100-500+/мес у агрегаторов. Платят только при результате.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ИИ-автоматизация</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Агрегаторы — витрины. Мы — агент-автопилот для клиента (заявки/мониторинг/документы).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Выравнивание интересов</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Мы зарабатываем ТОЛЬКО на закрытых сделках — стимул доводить клиента до подписания, а не продавать клики.</t>
+          <t>Публичные витрины; соблюдать ToS-риски. Эксклюзивы снижают зависимость от парсинга.</t>
         </is>
       </c>
     </row>
@@ -766,7 +639,7 @@
   <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -783,44 +656,44 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Инвестиция: $50K. Потрачено на запуск: $30K. Резерв на запуск/маркетинг: $20K.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Инвестиция: $50,000. Потрачено на запуск: $30,000. Резерв: $20,000.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -829,7 +702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Development (контракторы: фронт/бэк/парсер)</t>
+          <t>Разработка (фронт / бэк / парсер)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -855,7 +728,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AI/LLM APIs (Claude/OpenAI: автоматизация, письма)</t>
+          <t>AI / LLM API (автоматизация, письма)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -881,7 +754,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Design / UX (Framer, ассеты, брендинг)</t>
+          <t>Дизайн / UX (Framer, ассеты, брендинг)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -907,7 +780,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Infrastructure (Vercel, серверы, CMS, Mapbox, Resend)</t>
+          <t>Инфраструктура (Vercel, серверы, CMS, Mapbox, Resend)</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -959,7 +832,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tools &amp; Software (GitHub, Figma, Workspace, прочее)</t>
+          <t>Tools &amp; Software</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -985,7 +858,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Legal &amp; Company (юрлицо, договоры, DPA-шаблоны)</t>
+          <t>Legal и юрлицо (договоры, DPA-шаблоны)</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1011,7 +884,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Domain &amp; Trademark (book.immo, TM)</t>
+          <t>Домен и товарный знак (book.immo, TM)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1037,7 +910,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pre-launch marketing (лендинг-тесты, SEO-контент)</t>
+          <t>Pre-launch маркетинг (лендинг-тесты, SEO)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1063,7 +936,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Misc / buffer</t>
+          <t>Прочее / буфер</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1087,40 +960,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="6">
         <f>SUM(B5:B14)</f>
         <v/>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="6">
         <f>SUM(C5:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="6">
         <f>SUM(D5:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="6">
         <f>SUM(E5:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="6">
         <f>SUM(F5:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="6">
         <f>SUM(G5:G14)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Что построено за $30K:</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Что построено:</t>
         </is>
       </c>
     </row>
@@ -1198,75 +1071,75 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Модель: комиссионный сплит с агентствами + B2C pay-per-result. Деньги только при закрытых сделках.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Модель: комиссионный сплит с агентствами + B2C pay-per-result.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr"/>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>YEAR</t>
         </is>
@@ -1516,7 +1389,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rental: agent fee EUR 2,200 x 27.5% share</t>
+          <t>Rental: agent fee x 27.5% share</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1526,7 +1399,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sale: agent fee EUR 12,000 x 20% share</t>
+          <t>Sale: agent fee x 20% share</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1759,60 +1632,60 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="6">
         <f>SUM(B18:B21)</f>
         <v/>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="6">
         <f>SUM(C18:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="6">
         <f>SUM(D18:D21)</f>
         <v/>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="6">
         <f>SUM(E18:E21)</f>
         <v/>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="6">
         <f>SUM(F18:F21)</f>
         <v/>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="6">
         <f>SUM(G18:G21)</f>
         <v/>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="6">
         <f>SUM(H18:H21)</f>
         <v/>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="6">
         <f>SUM(I18:I21)</f>
         <v/>
       </c>
-      <c r="J22" s="8">
+      <c r="J22" s="6">
         <f>SUM(J18:J21)</f>
         <v/>
       </c>
-      <c r="K22" s="8">
+      <c r="K22" s="6">
         <f>SUM(K18:K21)</f>
         <v/>
       </c>
-      <c r="L22" s="8">
+      <c r="L22" s="6">
         <f>SUM(L18:L21)</f>
         <v/>
       </c>
-      <c r="M22" s="8">
+      <c r="M22" s="6">
         <f>SUM(M18:M21)</f>
         <v/>
       </c>
-      <c r="N22" s="8">
+      <c r="N22" s="6">
         <f>SUM(B22:M22)</f>
         <v/>
       </c>
@@ -1827,7 +1700,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Marketing B2C (perf + content + SEO)</t>
+          <t>Маркетинг B2C (performance + контент + SEO)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1870,7 +1743,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Agency sales / partnerships (part-time BD)</t>
+          <t>Продажи агентствам / партнёрства (part-time BD)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1913,7 +1786,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Team: dev/support (контракторы)</t>
+          <t>Команда: dev/support (контракторы)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1956,7 +1829,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Infrastructure + AI APIs</t>
+          <t>Инфраструктура + AI API</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1999,7 +1872,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tools, legal, misc</t>
+          <t>Tools, legal, прочее</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2040,66 +1913,66 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>TOTAL COSTS</t>
         </is>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="6">
         <f>SUM(B25:B29)</f>
         <v/>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="6">
         <f>SUM(C25:C29)</f>
         <v/>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="6">
         <f>SUM(D25:D29)</f>
         <v/>
       </c>
-      <c r="E30" s="8">
+      <c r="E30" s="6">
         <f>SUM(E25:E29)</f>
         <v/>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="6">
         <f>SUM(F25:F29)</f>
         <v/>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="6">
         <f>SUM(G25:G29)</f>
         <v/>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="6">
         <f>SUM(H25:H29)</f>
         <v/>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="6">
         <f>SUM(I25:I29)</f>
         <v/>
       </c>
-      <c r="J30" s="8">
+      <c r="J30" s="6">
         <f>SUM(J25:J29)</f>
         <v/>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="6">
         <f>SUM(K25:K29)</f>
         <v/>
       </c>
-      <c r="L30" s="8">
+      <c r="L30" s="6">
         <f>SUM(L25:L29)</f>
         <v/>
       </c>
-      <c r="M30" s="8">
+      <c r="M30" s="6">
         <f>SUM(M25:M29)</f>
         <v/>
       </c>
-      <c r="N30" s="8">
+      <c r="N30" s="6">
         <f>SUM(B30:M30)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
@@ -2160,7 +2033,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CUMULATIVE (incl. $20K reserve)</t>
+          <t>CUMULATIVE (incl. €18,000 reserve)</t>
         </is>
       </c>
       <c r="B33">
@@ -2213,9 +2086,9 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Note: R3 оформлен как оплата ИИ-сервиса (не Vermittlung) — см. лист Business Model / Legal.</t>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Note: R3 оформлен как оплата ИИ-сервиса (не Vermittlung) — см. лист Business Model.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify SEO channel: acquisition source vs deal source
The card read as a contradiction: "catalogue isn't for deals" next
to "19% of qualified leads." Channel = how someone finds us; once
inside, they see both the catalogue and agency exclusives, so most
still close via an exclusive, not the listing that brought them in.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plan/bookimmo_business_plan_v2.xlsx
+++ b/public/plan/bookimmo_business_plan_v2.xlsx
@@ -586,12 +586,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SEO на каталоге IS24/Immowelt</t>
+          <t>SEO: гео-страницы на базе каталога</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 40%] Страницы район × комнаты × бюджет, DE + EN. Каталог IS24 — для полноты и трафика, не для сделок: туда доходят остатки, не разобранные внутри CRM агентств.</t>
+          <t>[квалификация 40%] Программные страницы район × комнаты × бюджет (DE + EN) на данных парсинга IS24/Immowelt — это как человек нас находит через поиск, а не то, что он снимет. Внутри у него доступ и к каталогу, и к эксклюзивам агентств — сам каталог для сделок слабый (остатки, не разобранные в CRM), но именно поэтому большинство таких лидов закрывается через эксклюзив, а не через объявление, которое их привело.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SEO на каталоге IS24/Immowelt</t>
+          <t xml:space="preserve">  SEO: гео-страницы на базе каталога</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
@@ -4097,7 +4097,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SEO на каталоге IS24/Immowelt</t>
+          <t xml:space="preserve">  SEO: гео-страницы на базе каталога</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">

</xml_diff>

<commit_message>
Break dev/support lump sum into 3 explicit roles
"Команда: dev/support (контракторы)" (EUR45K/year) was a single
unexplained number. Split into backend contractor (60%), parser/
infra maintenance -- IS24 anti-bot changes, Chrome pipeline fixes
(20%), and support/ops for both B2C users and agencies (20%).
Totals per month unchanged, so revenue/EBITDA/breakeven are
identical -- this is pure transparency, not a cost change. Both
/plan (deck, via channel-cost averages) and /plan/text (growth
budget breakdown) read this from the same JSON, so both updated
automatically.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plan/bookimmo_business_plan_v2.xlsx
+++ b/public/plan/bookimmo_business_plan_v2.xlsx
@@ -1149,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3299,44 +3299,44 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Команда: dev / support (контракторы)</t>
+          <t>Backend-контрактор (доработки, фичи)</t>
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="C73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="D73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="G73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="I73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="J73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="K73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="L73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="M73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="N73">
         <f>SUM(B73:M73)</f>
@@ -3346,44 +3346,44 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Инфраструктура + AI API</t>
+          <t>Парсер / инфра-мейнтенанс (IS24 anti-bot, Chrome pipeline)</t>
         </is>
       </c>
       <c r="B74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="C74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="E74" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="C74" s="8" t="n">
-        <v>750</v>
-      </c>
-      <c r="D74" s="8" t="n">
+      <c r="F74" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="H74" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="E74" s="8" t="n">
-        <v>850</v>
-      </c>
-      <c r="F74" s="8" t="n">
+      <c r="I74" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="J74" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="K74" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="G74" s="8" t="n">
-        <v>950</v>
-      </c>
-      <c r="H74" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I74" s="8" t="n">
-        <v>1050</v>
-      </c>
-      <c r="J74" s="8" t="n">
-        <v>1100</v>
-      </c>
-      <c r="K74" s="8" t="n">
-        <v>1150</v>
-      </c>
       <c r="L74" s="8" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="M74" s="8" t="n">
-        <v>1250</v>
+        <v>900</v>
       </c>
       <c r="N74">
         <f>SUM(B74:M74)</f>
@@ -3393,44 +3393,44 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tools, legal, прочее</t>
+          <t>Support/ops (B2C + агентства)</t>
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="C75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="G75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="J75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="K75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="L75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="M75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="N75">
         <f>SUM(B75:M75)</f>
@@ -3440,56 +3440,44 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Продажник: комиссия (% от R1+R2)</t>
-        </is>
-      </c>
-      <c r="B76">
-        <f>ROUND(B63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="C76">
-        <f>ROUND(C63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="D76">
-        <f>ROUND(D63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="E76">
-        <f>ROUND(E63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="F76">
-        <f>ROUND(F63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="G76">
-        <f>ROUND(G63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="H76">
-        <f>ROUND(H63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="I76">
-        <f>ROUND(I63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="J76">
-        <f>ROUND(J63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="K76">
-        <f>ROUND(K63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="L76">
-        <f>ROUND(L63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="M76">
-        <f>ROUND(M63*$B$38,0)</f>
-        <v/>
+          <t>Инфраструктура + AI API</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="C76" s="8" t="n">
+        <v>750</v>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="F76" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>950</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I76" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="J76" s="8" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K76" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="L76" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M76" s="8" t="n">
+        <v>1250</v>
       </c>
       <c r="N76">
         <f>SUM(B76:M76)</f>
@@ -3497,116 +3485,163 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL COSTS</t>
-        </is>
-      </c>
-      <c r="B77" s="6">
-        <f>B70+B71+B72+B73+B74+B75+B76</f>
-        <v/>
-      </c>
-      <c r="C77" s="6">
-        <f>C70+C71+C72+C73+C74+C75+C76</f>
-        <v/>
-      </c>
-      <c r="D77" s="6">
-        <f>D70+D71+D72+D73+D74+D75+D76</f>
-        <v/>
-      </c>
-      <c r="E77" s="6">
-        <f>E70+E71+E72+E73+E74+E75+E76</f>
-        <v/>
-      </c>
-      <c r="F77" s="6">
-        <f>F70+F71+F72+F73+F74+F75+F76</f>
-        <v/>
-      </c>
-      <c r="G77" s="6">
-        <f>G70+G71+G72+G73+G74+G75+G76</f>
-        <v/>
-      </c>
-      <c r="H77" s="6">
-        <f>H70+H71+H72+H73+H74+H75+H76</f>
-        <v/>
-      </c>
-      <c r="I77" s="6">
-        <f>I70+I71+I72+I73+I74+I75+I76</f>
-        <v/>
-      </c>
-      <c r="J77" s="6">
-        <f>J70+J71+J72+J73+J74+J75+J76</f>
-        <v/>
-      </c>
-      <c r="K77" s="6">
-        <f>K70+K71+K72+K73+K74+K75+K76</f>
-        <v/>
-      </c>
-      <c r="L77" s="6">
-        <f>L70+L71+L72+L73+L74+L75+L76</f>
-        <v/>
-      </c>
-      <c r="M77" s="6">
-        <f>M70+M71+M72+M73+M74+M75+M76</f>
-        <v/>
-      </c>
-      <c r="N77" s="6">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Tools, legal, прочее</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="J77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="K77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="L77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="M77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="N77">
         <f>SUM(B77:M77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Продажник: комиссия (% от R1+R2)</t>
+        </is>
+      </c>
+      <c r="B78">
+        <f>ROUND(B63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="C78">
+        <f>ROUND(C63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="D78">
+        <f>ROUND(D63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="E78">
+        <f>ROUND(E63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="F78">
+        <f>ROUND(F63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="G78">
+        <f>ROUND(G63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="H78">
+        <f>ROUND(H63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="I78">
+        <f>ROUND(I63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="J78">
+        <f>ROUND(J63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="K78">
+        <f>ROUND(K63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="L78">
+        <f>ROUND(L63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="M78">
+        <f>ROUND(M63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="N78">
+        <f>SUM(B78:M78)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>TOTAL COSTS</t>
         </is>
       </c>
       <c r="B79" s="6">
-        <f>B67-B77</f>
+        <f>B70+B71+B72+B73+B74+B75+B76+B77+B78</f>
         <v/>
       </c>
       <c r="C79" s="6">
-        <f>C67-C77</f>
+        <f>C70+C71+C72+C73+C74+C75+C76+C77+C78</f>
         <v/>
       </c>
       <c r="D79" s="6">
-        <f>D67-D77</f>
+        <f>D70+D71+D72+D73+D74+D75+D76+D77+D78</f>
         <v/>
       </c>
       <c r="E79" s="6">
-        <f>E67-E77</f>
+        <f>E70+E71+E72+E73+E74+E75+E76+E77+E78</f>
         <v/>
       </c>
       <c r="F79" s="6">
-        <f>F67-F77</f>
+        <f>F70+F71+F72+F73+F74+F75+F76+F77+F78</f>
         <v/>
       </c>
       <c r="G79" s="6">
-        <f>G67-G77</f>
+        <f>G70+G71+G72+G73+G74+G75+G76+G77+G78</f>
         <v/>
       </c>
       <c r="H79" s="6">
-        <f>H67-H77</f>
+        <f>H70+H71+H72+H73+H74+H75+H76+H77+H78</f>
         <v/>
       </c>
       <c r="I79" s="6">
-        <f>I67-I77</f>
+        <f>I70+I71+I72+I73+I74+I75+I76+I77+I78</f>
         <v/>
       </c>
       <c r="J79" s="6">
-        <f>J67-J77</f>
+        <f>J70+J71+J72+J73+J74+J75+J76+J77+J78</f>
         <v/>
       </c>
       <c r="K79" s="6">
-        <f>K67-K77</f>
+        <f>K70+K71+K72+K73+K74+K75+K76+K77+K78</f>
         <v/>
       </c>
       <c r="L79" s="6">
-        <f>L67-L77</f>
+        <f>L70+L71+L72+L73+L74+L75+L76+L77+L78</f>
         <v/>
       </c>
       <c r="M79" s="6">
-        <f>M67-M77</f>
+        <f>M70+M71+M72+M73+M74+M75+M76+M77+M78</f>
         <v/>
       </c>
       <c r="N79" s="6">
@@ -3614,109 +3649,168 @@
         <v/>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B81" s="6">
+        <f>B67-B79</f>
+        <v/>
+      </c>
+      <c r="C81" s="6">
+        <f>C67-C79</f>
+        <v/>
+      </c>
+      <c r="D81" s="6">
+        <f>D67-D79</f>
+        <v/>
+      </c>
+      <c r="E81" s="6">
+        <f>E67-E79</f>
+        <v/>
+      </c>
+      <c r="F81" s="6">
+        <f>F67-F79</f>
+        <v/>
+      </c>
+      <c r="G81" s="6">
+        <f>G67-G79</f>
+        <v/>
+      </c>
+      <c r="H81" s="6">
+        <f>H67-H79</f>
+        <v/>
+      </c>
+      <c r="I81" s="6">
+        <f>I67-I79</f>
+        <v/>
+      </c>
+      <c r="J81" s="6">
+        <f>J67-J79</f>
+        <v/>
+      </c>
+      <c r="K81" s="6">
+        <f>K67-K79</f>
+        <v/>
+      </c>
+      <c r="L81" s="6">
+        <f>L67-L79</f>
+        <v/>
+      </c>
+      <c r="M81" s="6">
+        <f>M67-M79</f>
+        <v/>
+      </c>
+      <c r="N81" s="6">
+        <f>SUM(B81:M81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>Кэш (старт €18,000)</t>
         </is>
       </c>
-      <c r="B80">
-        <f>18000+B79</f>
-        <v/>
-      </c>
-      <c r="C80">
-        <f>B80+C79</f>
-        <v/>
-      </c>
-      <c r="D80">
-        <f>C80+D79</f>
-        <v/>
-      </c>
-      <c r="E80">
-        <f>D80+E79</f>
-        <v/>
-      </c>
-      <c r="F80">
-        <f>E80+F79</f>
-        <v/>
-      </c>
-      <c r="G80">
-        <f>F80+G79</f>
-        <v/>
-      </c>
-      <c r="H80">
-        <f>G80+H79</f>
-        <v/>
-      </c>
-      <c r="I80">
-        <f>H80+I79</f>
-        <v/>
-      </c>
-      <c r="J80">
-        <f>I80+J79</f>
-        <v/>
-      </c>
-      <c r="K80">
-        <f>J80+K79</f>
-        <v/>
-      </c>
-      <c r="L80">
-        <f>K80+L79</f>
-        <v/>
-      </c>
-      <c r="M80">
-        <f>L80+M79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+      <c r="B82">
+        <f>18000+B81</f>
+        <v/>
+      </c>
+      <c r="C82">
+        <f>B82+C81</f>
+        <v/>
+      </c>
+      <c r="D82">
+        <f>C82+D81</f>
+        <v/>
+      </c>
+      <c r="E82">
+        <f>D82+E81</f>
+        <v/>
+      </c>
+      <c r="F82">
+        <f>E82+F81</f>
+        <v/>
+      </c>
+      <c r="G82">
+        <f>F82+G81</f>
+        <v/>
+      </c>
+      <c r="H82">
+        <f>G82+H81</f>
+        <v/>
+      </c>
+      <c r="I82">
+        <f>H82+I81</f>
+        <v/>
+      </c>
+      <c r="J82">
+        <f>I82+J81</f>
+        <v/>
+      </c>
+      <c r="K82">
+        <f>J82+K81</f>
+        <v/>
+      </c>
+      <c r="L82">
+        <f>K82+L81</f>
+        <v/>
+      </c>
+      <c r="M82">
+        <f>L82+M81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>ЮНИТ-ЭКОНОМИКА (год)</t>
         </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>CAC на квалифицированного лида, €</t>
-        </is>
-      </c>
-      <c r="B83">
-        <f>ROUND(N6/N56,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>CAC на сделку, €</t>
-        </is>
-      </c>
-      <c r="B84">
-        <f>ROUND(N6/N59,0)</f>
-        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Выручка на агентскую сделку, €</t>
+          <t>CAC на квалифицированного лида, €</t>
         </is>
       </c>
       <c r="B85">
-        <f>ROUND($B$35*$B$33+(1-$B$35)*$B$34,0)</f>
+        <f>ROUND(N6/N56,0)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>CAC на сделку, €</t>
+        </is>
+      </c>
+      <c r="B86">
+        <f>ROUND(N6/N59,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Выручка на агентскую сделку, €</t>
+        </is>
+      </c>
+      <c r="B87">
+        <f>ROUND($B$35*$B$33+(1-$B$35)*$B$34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>LTV / CAC (агентский канал)</t>
         </is>
       </c>
-      <c r="B86">
-        <f>ROUND(B85/B84,1)</f>
+      <c r="B88">
+        <f>ROUND(B87/B86,1)</f>
         <v/>
       </c>
     </row>
@@ -3731,7 +3825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -5881,44 +5975,44 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Команда: dev / support (контракторы)</t>
+          <t>Backend-контрактор (доработки, фичи)</t>
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="C73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="D73" s="8" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="G73" s="8" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="I73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="J73" s="8" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="K73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="L73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="M73" s="8" t="n">
-        <v>4500</v>
+        <v>2700</v>
       </c>
       <c r="N73">
         <f>SUM(B73:M73)</f>
@@ -5928,44 +6022,44 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Инфраструктура + AI API</t>
+          <t>Парсер / инфра-мейнтенанс (IS24 anti-bot, Chrome pipeline)</t>
         </is>
       </c>
       <c r="B74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="C74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="E74" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="C74" s="8" t="n">
-        <v>750</v>
-      </c>
-      <c r="D74" s="8" t="n">
+      <c r="F74" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="H74" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="E74" s="8" t="n">
-        <v>850</v>
-      </c>
-      <c r="F74" s="8" t="n">
+      <c r="I74" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="J74" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="K74" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="G74" s="8" t="n">
-        <v>950</v>
-      </c>
-      <c r="H74" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I74" s="8" t="n">
-        <v>1050</v>
-      </c>
-      <c r="J74" s="8" t="n">
-        <v>1100</v>
-      </c>
-      <c r="K74" s="8" t="n">
-        <v>1150</v>
-      </c>
       <c r="L74" s="8" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="M74" s="8" t="n">
-        <v>1250</v>
+        <v>900</v>
       </c>
       <c r="N74">
         <f>SUM(B74:M74)</f>
@@ -5975,44 +6069,44 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tools, legal, прочее</t>
+          <t>Support/ops (B2C + агентства)</t>
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="C75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="G75" s="8" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="J75" s="8" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="K75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="L75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="M75" s="8" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="N75">
         <f>SUM(B75:M75)</f>
@@ -6022,56 +6116,44 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Продажник: комиссия (% от R1+R2)</t>
-        </is>
-      </c>
-      <c r="B76">
-        <f>ROUND(B63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="C76">
-        <f>ROUND(C63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="D76">
-        <f>ROUND(D63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="E76">
-        <f>ROUND(E63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="F76">
-        <f>ROUND(F63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="G76">
-        <f>ROUND(G63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="H76">
-        <f>ROUND(H63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="I76">
-        <f>ROUND(I63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="J76">
-        <f>ROUND(J63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="K76">
-        <f>ROUND(K63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="L76">
-        <f>ROUND(L63*$B$38,0)</f>
-        <v/>
-      </c>
-      <c r="M76">
-        <f>ROUND(M63*$B$38,0)</f>
-        <v/>
+          <t>Инфраструктура + AI API</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="C76" s="8" t="n">
+        <v>750</v>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="F76" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>950</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I76" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="J76" s="8" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K76" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="L76" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M76" s="8" t="n">
+        <v>1250</v>
       </c>
       <c r="N76">
         <f>SUM(B76:M76)</f>
@@ -6079,116 +6161,163 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL COSTS</t>
-        </is>
-      </c>
-      <c r="B77" s="6">
-        <f>B70+B71+B72+B73+B74+B75+B76</f>
-        <v/>
-      </c>
-      <c r="C77" s="6">
-        <f>C70+C71+C72+C73+C74+C75+C76</f>
-        <v/>
-      </c>
-      <c r="D77" s="6">
-        <f>D70+D71+D72+D73+D74+D75+D76</f>
-        <v/>
-      </c>
-      <c r="E77" s="6">
-        <f>E70+E71+E72+E73+E74+E75+E76</f>
-        <v/>
-      </c>
-      <c r="F77" s="6">
-        <f>F70+F71+F72+F73+F74+F75+F76</f>
-        <v/>
-      </c>
-      <c r="G77" s="6">
-        <f>G70+G71+G72+G73+G74+G75+G76</f>
-        <v/>
-      </c>
-      <c r="H77" s="6">
-        <f>H70+H71+H72+H73+H74+H75+H76</f>
-        <v/>
-      </c>
-      <c r="I77" s="6">
-        <f>I70+I71+I72+I73+I74+I75+I76</f>
-        <v/>
-      </c>
-      <c r="J77" s="6">
-        <f>J70+J71+J72+J73+J74+J75+J76</f>
-        <v/>
-      </c>
-      <c r="K77" s="6">
-        <f>K70+K71+K72+K73+K74+K75+K76</f>
-        <v/>
-      </c>
-      <c r="L77" s="6">
-        <f>L70+L71+L72+L73+L74+L75+L76</f>
-        <v/>
-      </c>
-      <c r="M77" s="6">
-        <f>M70+M71+M72+M73+M74+M75+M76</f>
-        <v/>
-      </c>
-      <c r="N77" s="6">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Tools, legal, прочее</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="J77" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="K77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="L77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="M77" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="N77">
         <f>SUM(B77:M77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Продажник: комиссия (% от R1+R2)</t>
+        </is>
+      </c>
+      <c r="B78">
+        <f>ROUND(B63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="C78">
+        <f>ROUND(C63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="D78">
+        <f>ROUND(D63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="E78">
+        <f>ROUND(E63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="F78">
+        <f>ROUND(F63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="G78">
+        <f>ROUND(G63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="H78">
+        <f>ROUND(H63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="I78">
+        <f>ROUND(I63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="J78">
+        <f>ROUND(J63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="K78">
+        <f>ROUND(K63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="L78">
+        <f>ROUND(L63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="M78">
+        <f>ROUND(M63*$B$38,0)</f>
+        <v/>
+      </c>
+      <c r="N78">
+        <f>SUM(B78:M78)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>TOTAL COSTS</t>
         </is>
       </c>
       <c r="B79" s="6">
-        <f>B67-B77</f>
+        <f>B70+B71+B72+B73+B74+B75+B76+B77+B78</f>
         <v/>
       </c>
       <c r="C79" s="6">
-        <f>C67-C77</f>
+        <f>C70+C71+C72+C73+C74+C75+C76+C77+C78</f>
         <v/>
       </c>
       <c r="D79" s="6">
-        <f>D67-D77</f>
+        <f>D70+D71+D72+D73+D74+D75+D76+D77+D78</f>
         <v/>
       </c>
       <c r="E79" s="6">
-        <f>E67-E77</f>
+        <f>E70+E71+E72+E73+E74+E75+E76+E77+E78</f>
         <v/>
       </c>
       <c r="F79" s="6">
-        <f>F67-F77</f>
+        <f>F70+F71+F72+F73+F74+F75+F76+F77+F78</f>
         <v/>
       </c>
       <c r="G79" s="6">
-        <f>G67-G77</f>
+        <f>G70+G71+G72+G73+G74+G75+G76+G77+G78</f>
         <v/>
       </c>
       <c r="H79" s="6">
-        <f>H67-H77</f>
+        <f>H70+H71+H72+H73+H74+H75+H76+H77+H78</f>
         <v/>
       </c>
       <c r="I79" s="6">
-        <f>I67-I77</f>
+        <f>I70+I71+I72+I73+I74+I75+I76+I77+I78</f>
         <v/>
       </c>
       <c r="J79" s="6">
-        <f>J67-J77</f>
+        <f>J70+J71+J72+J73+J74+J75+J76+J77+J78</f>
         <v/>
       </c>
       <c r="K79" s="6">
-        <f>K67-K77</f>
+        <f>K70+K71+K72+K73+K74+K75+K76+K77+K78</f>
         <v/>
       </c>
       <c r="L79" s="6">
-        <f>L67-L77</f>
+        <f>L70+L71+L72+L73+L74+L75+L76+L77+L78</f>
         <v/>
       </c>
       <c r="M79" s="6">
-        <f>M67-M77</f>
+        <f>M70+M71+M72+M73+M74+M75+M76+M77+M78</f>
         <v/>
       </c>
       <c r="N79" s="6">
@@ -6196,109 +6325,168 @@
         <v/>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B81" s="6">
+        <f>B67-B79</f>
+        <v/>
+      </c>
+      <c r="C81" s="6">
+        <f>C67-C79</f>
+        <v/>
+      </c>
+      <c r="D81" s="6">
+        <f>D67-D79</f>
+        <v/>
+      </c>
+      <c r="E81" s="6">
+        <f>E67-E79</f>
+        <v/>
+      </c>
+      <c r="F81" s="6">
+        <f>F67-F79</f>
+        <v/>
+      </c>
+      <c r="G81" s="6">
+        <f>G67-G79</f>
+        <v/>
+      </c>
+      <c r="H81" s="6">
+        <f>H67-H79</f>
+        <v/>
+      </c>
+      <c r="I81" s="6">
+        <f>I67-I79</f>
+        <v/>
+      </c>
+      <c r="J81" s="6">
+        <f>J67-J79</f>
+        <v/>
+      </c>
+      <c r="K81" s="6">
+        <f>K67-K79</f>
+        <v/>
+      </c>
+      <c r="L81" s="6">
+        <f>L67-L79</f>
+        <v/>
+      </c>
+      <c r="M81" s="6">
+        <f>M67-M79</f>
+        <v/>
+      </c>
+      <c r="N81" s="6">
+        <f>SUM(B81:M81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>Кэш (старт €18,000)</t>
         </is>
       </c>
-      <c r="B80">
-        <f>18000+B79</f>
-        <v/>
-      </c>
-      <c r="C80">
-        <f>B80+C79</f>
-        <v/>
-      </c>
-      <c r="D80">
-        <f>C80+D79</f>
-        <v/>
-      </c>
-      <c r="E80">
-        <f>D80+E79</f>
-        <v/>
-      </c>
-      <c r="F80">
-        <f>E80+F79</f>
-        <v/>
-      </c>
-      <c r="G80">
-        <f>F80+G79</f>
-        <v/>
-      </c>
-      <c r="H80">
-        <f>G80+H79</f>
-        <v/>
-      </c>
-      <c r="I80">
-        <f>H80+I79</f>
-        <v/>
-      </c>
-      <c r="J80">
-        <f>I80+J79</f>
-        <v/>
-      </c>
-      <c r="K80">
-        <f>J80+K79</f>
-        <v/>
-      </c>
-      <c r="L80">
-        <f>K80+L79</f>
-        <v/>
-      </c>
-      <c r="M80">
-        <f>L80+M79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+      <c r="B82">
+        <f>18000+B81</f>
+        <v/>
+      </c>
+      <c r="C82">
+        <f>B82+C81</f>
+        <v/>
+      </c>
+      <c r="D82">
+        <f>C82+D81</f>
+        <v/>
+      </c>
+      <c r="E82">
+        <f>D82+E81</f>
+        <v/>
+      </c>
+      <c r="F82">
+        <f>E82+F81</f>
+        <v/>
+      </c>
+      <c r="G82">
+        <f>F82+G81</f>
+        <v/>
+      </c>
+      <c r="H82">
+        <f>G82+H81</f>
+        <v/>
+      </c>
+      <c r="I82">
+        <f>H82+I81</f>
+        <v/>
+      </c>
+      <c r="J82">
+        <f>I82+J81</f>
+        <v/>
+      </c>
+      <c r="K82">
+        <f>J82+K81</f>
+        <v/>
+      </c>
+      <c r="L82">
+        <f>K82+L81</f>
+        <v/>
+      </c>
+      <c r="M82">
+        <f>L82+M81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>ЮНИТ-ЭКОНОМИКА (год)</t>
         </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>CAC на квалифицированного лида, €</t>
-        </is>
-      </c>
-      <c r="B83">
-        <f>ROUND(N6/N56,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>CAC на сделку, €</t>
-        </is>
-      </c>
-      <c r="B84">
-        <f>ROUND(N6/N59,0)</f>
-        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Выручка на агентскую сделку, €</t>
+          <t>CAC на квалифицированного лида, €</t>
         </is>
       </c>
       <c r="B85">
-        <f>ROUND($B$35*$B$33+(1-$B$35)*$B$34,0)</f>
+        <f>ROUND(N6/N56,0)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>CAC на сделку, €</t>
+        </is>
+      </c>
+      <c r="B86">
+        <f>ROUND(N6/N59,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Выручка на агентскую сделку, €</t>
+        </is>
+      </c>
+      <c r="B87">
+        <f>ROUND($B$35*$B$33+(1-$B$35)*$B$34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>LTV / CAC (агентский канал)</t>
         </is>
       </c>
-      <c r="B86">
-        <f>ROUND(B85/B84,1)</f>
+      <c r="B88">
+        <f>ROUND(B87/B86,1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix overlapping text on the lead-channels slide, trim xlsx generation
The slide had 6 channel cards plus a summary line plus a redundant
bottom note — more content than the fixed-height slide could hold,
so the second row of cards visually overlapped the bottom note.
Trimmed every channel description to one short sentence, dropped
the redundant bottom note (its point was already in the sub line),
shortened the per-card cost labels, and added scoped smaller font
sizes for this slide's heading/sub/cards. Verified no overflow via
actual getBoundingClientRect() checks, not just a screenshot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plan/bookimmo_business_plan_v2.xlsx
+++ b/public/plan/bookimmo_business_plan_v2.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 35%] Только узкие запросы («Wohnung Berlin ohne Schufa», «apartment berlin english») и ретаргетинг. Кран, а не основа.</t>
+          <t>[квалификация 35%] Узкие запросы и ретаргетинг. Кран, а не основа.</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 22%] FB «Berlin Housing», r/berlin, Telegram, Toytown. Дёшево и горячо, но часто нет немецких документов о доходе — квалификация ~22%. Для них шаг «доведение документов»: Bürgschaft, письмо работодателя, Schufa через нас.</t>
+          <t>[квалификация 22%] FB, r/berlin, Telegram. Дёшево, но часто без немецких доходных справок.</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 100%] HR берлинских стартапов, международные офисы TU/HU/FU, буткемпы. Приходят с датой въезда и подтверждённым работодателем доходом — уже квалифицированы.</t>
+          <t>[квалификация 100%] HR стартапов, вузы. Приходят с датой въезда и доходом — уже квалифицированы.</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 40%] Программные страницы район × комнаты × бюджет (DE + EN) на данных парсинга IS24/Immowelt — это как человек нас находит через поиск, а не то, что он снимет. Внутри у него доступ и к каталогу, и к эксклюзивам агентств — сам каталог для сделок слабый (остатки, не разобранные в CRM), но именно поэтому большинство таких лидов закрывается через эксклюзив, а не через объявление, которое их привело.</t>
+          <t>[квалификация 40%] Гео-страницы на данных парсинга — способ найти нас, а не ограничение на сделку: внутри доступны и каталог, и эксклюзивы.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 50%] Каждый заселённый знает пятерых ищущих. Бесплатный месяц мониторинга за приведённого, кто подписал.</t>
+          <t>[квалификация 50%] Заселённый клиент приводит следующего — месяц мониторинга в подарок.</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 50%] Эксклюзивы из CRM в топе выдачи + агентства шлют свои waiting-list'ы на страницу объекта у нас. Интент на конкретную квартиру.</t>
+          <t>[квалификация 50%] Эксклюзивы в топе выдачи + агентства шлют свой waiting-list к нам.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align revenue-stream cards on shared baselines, remove all em-dashes
- .gcard-t gets a fixed min-height (2 lines) so title, price and
  description rows start at identical Y across every card in a row,
  regardless of how many lines a given title wraps to (verified via
  getBoundingClientRect(), not just a screenshot)
- Replaced every em-dash (—) across the deck, text plan, shared
  JSON, and the xlsx generator with a plain hyphen, per house style

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plan/bookimmo_business_plan_v2.xlsx
+++ b/public/plan/bookimmo_business_plan_v2.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Model" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget Apr-Aug (USD)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE — Берлин" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PESSIMISTIC — Берлин" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE - Берлин" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PESSIMISTIC - Берлин" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>book.immo — Business Model v2</t>
+          <t>book.immo - Business Model v2</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Берлин — стартовый рынок, затем другие города Германии</t>
+          <t>Берлин - стартовый рынок, затем другие города Германии</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRM агентства выгружает на IS24 то, что не ушло по своей базе. Хорошие объекты на витрину не доходят. book.immo получает их из CRM до публикации — бесплатно для агентства, за сплит комиссии при сделке.</t>
+          <t>CRM агентства выгружает на IS24 то, что не ушло по своей базе. Хорошие объекты на витрину не доходят. book.immo получает их из CRM до публикации - бесплатно для агентства, за сплит комиссии при сделке.</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Парсинг — для полноты каталога и SEO-трафика, не для сделок: там остатки.</t>
+          <t>Парсинг - для полноты каталога и SEO-трафика, не для сделок: там остатки.</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 100%] HR стартапов, вузы. Приходят с датой въезда и доходом — уже квалифицированы.</t>
+          <t>[квалификация 100%] HR стартапов, вузы. Приходят с датой въезда и доходом - уже квалифицированы.</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 40%] Гео-страницы на данных парсинга — способ найти нас, а не ограничение на сделку: внутри доступны и каталог, и эксклюзивы.</t>
+          <t>[квалификация 40%] Гео-страницы на данных парсинга - способ найти нас, а не ограничение на сделку: внутри доступны и каталог, и эксклюзивы.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>[квалификация 50%] Заселённый клиент приводит следующего — месяц мониторинга в подарок.</t>
+          <t>[квалификация 50%] Заселённый клиент приводит следующего - месяц мониторинга в подарок.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Бесплатный ИИ-пакет документов: доход, состав семьи, дата въезда вводятся, чтобы его получить — квалификация на входе</t>
+          <t>Бесплатный ИИ-пакет документов: доход, состав семьи, дата въезда вводятся, чтобы его получить - квалификация на входе</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Schufa-готовность, доход ≥ 3× Kaltmiete. Экспатам без немецких справок — Bürgschaft/гарант, письмо работодателя, Schufa через нас</t>
+          <t>Schufa-готовность, доход ≥ 3× Kaltmiete. Экспатам без немецких справок - Bürgschaft/гарант, письмо работодателя, Schufa через нас</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Монитор + полный пакет → подача сразу после публикации. На эксклюзивы агентств — приоритетно, на каталог IS24 — как страховка</t>
+          <t>Монитор + полный пакет → подача сразу после публикации. На эксклюзивы агентств - приоритетно, на каталог IS24 - как страховка</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Только квалифицированные и только под конкретный эксклюзив — агентство не тратит время на шум</t>
+          <t>Только квалифицированные и только под конкретный эксклюзив - агентство не тратит время на шум</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Подписание через агентство (сплит комиссии). Закрытия на остатках IS24 — редкие, только B2C fee</t>
+          <t>Подписание через агентство (сплит комиссии). Закрытия на остатках IS24 - редкие, только B2C fee</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Нельзя брать с арендатора комиссию за посредничество. B2C fee — плата за софт (автозаявки, мониторинг, документы). Нужен письменный legal opinion до запуска.</t>
+          <t>Нельзя брать с арендатора комиссию за посредничество. B2C fee - плата за софт (автозаявки, мониторинг, документы). Нужен письменный legal opinion до запуска.</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Комиссию платит собственник маклеру. Сплит book.immo — из B2B-агентского договора. Легально.</t>
+          <t>Комиссию платит собственник маклеру. Сплит book.immo - из B2B-агентского договора. Легально.</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>book.immo — Pre-Launch Budget (Apr–Aug 2026, USD)</t>
+          <t>book.immo - Pre-Launch Budget (Apr–Aug 2026, USD)</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>• Собственный бэкенд: PostgreSQL + API (auth, избранное, заявки) — без vendor lock-in</t>
+          <t>• Собственный бэкенд: PostgreSQL + API (auth, избранное, заявки) - без vendor lock-in</t>
         </is>
       </c>
     </row>
@@ -1171,14 +1171,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>book.immo — BASE, Берлин, запуск Sep 2026 (EUR)</t>
+          <t>book.immo - BASE, Берлин, запуск Sep 2026 (EUR)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки — входные драйверы (можно менять). Остальное считается формулами.</t>
+          <t>Жёлтые ячейки - входные драйверы (можно менять). Остальное считается формулами.</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ДРАЙВЕРЫ — каналы (входные)</t>
+          <t>ДРАЙВЕРЫ - каналы (входные)</t>
         </is>
       </c>
     </row>
@@ -3847,14 +3847,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>book.immo — PESSIMISTIC, Берлин, запуск Sep 2026 (EUR)</t>
+          <t>book.immo - PESSIMISTIC, Берлин, запуск Sep 2026 (EUR)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки — входные драйверы (можно менять). Остальное считается формулами.</t>
+          <t>Жёлтые ячейки - входные драйверы (можно менять). Остальное считается формулами.</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ДРАЙВЕРЫ — каналы (входные)</t>
+          <t>ДРАЙВЕРЫ - каналы (входные)</t>
         </is>
       </c>
     </row>

</xml_diff>